<commit_message>
Additional notes to the SpD annotation
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k09.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k09.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{43B4E268-D601-DD4F-ADCC-94FE2ACA6991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1661A0A0-F92B-EB49-BD5C-7C862AF1AAA8}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{43B4E268-D601-DD4F-ADCC-94FE2ACA6991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5613757C-247F-0742-A754-37472DAB709C}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="26440" windowHeight="9880" xr2:uid="{122630C5-77A4-D449-8A1A-052F0B5B4F44}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="26440" windowHeight="11180" xr2:uid="{122630C5-77A4-D449-8A1A-052F0B5B4F44}"/>
   </bookViews>
   <sheets>
     <sheet name="ERC_SpD_spatial_registration_an" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ERC_SpD_spatial_registration_an!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
   <si>
     <t>cluster</t>
   </si>
@@ -164,6 +164,36 @@
   </si>
   <si>
     <t>WMuf</t>
+  </si>
+  <si>
+    <t>Xenium_SpX</t>
+  </si>
+  <si>
+    <t>L2.3~SpX4</t>
+  </si>
+  <si>
+    <t>Inhib~SpX5/L2.3~SpX4/L1b~SpX7/L5~SpX1</t>
+  </si>
+  <si>
+    <t>L5~SpX1</t>
+  </si>
+  <si>
+    <t>L6~SpX9</t>
+  </si>
+  <si>
+    <t>L1b~SpX7/L1a~SpX6</t>
+  </si>
+  <si>
+    <t>WM~SpX2/L1a~SpX6</t>
+  </si>
+  <si>
+    <t>WM~SpX2</t>
+  </si>
+  <si>
+    <t>Vasc~SpX3</t>
+  </si>
+  <si>
+    <t>L5~SpX1/L2.3~SpX4</t>
   </si>
 </sst>
 </file>
@@ -705,6 +735,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1024,17 +1058,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2586EF44-A1D0-B145-AA11-6BC6F33FD8C1}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="90.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="37.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1048,198 +1083,223 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B9" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C9" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D9" t="s">
         <v>7</v>
       </c>
-      <c r="E2">
+      <c r="E9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
-      </c>
-      <c r="F5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C10" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="E6">
+      <c r="E10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10">
         <v>4</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G10" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8">
-        <v>6</v>
-      </c>
-      <c r="F8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9">
-        <v>7</v>
-      </c>
-      <c r="F9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10">
-        <v>8</v>
-      </c>
-      <c r="F10" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{2586EF44-A1D0-B145-AA11-6BC6F33FD8C1}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F10">
-      <sortCondition ref="E1:E10"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix lables and colnames
</commit_message>
<xml_diff>
--- a/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k09.xlsx
+++ b/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/ERC_SpD_spatial_registration_anno_summary_k09.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/05_spe_correct_cluster/10_spatial_registration_DLPFC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{43B4E268-D601-DD4F-ADCC-94FE2ACA6991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E6E3637-D290-DF4C-8BC7-A9F771B878EB}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{43B4E268-D601-DD4F-ADCC-94FE2ACA6991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46BA05CF-B559-CB4F-81FE-ABE984D6922E}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="26440" windowHeight="11180" xr2:uid="{122630C5-77A4-D449-8A1A-052F0B5B4F44}"/>
+    <workbookView xWindow="-27760" yWindow="-26240" windowWidth="26440" windowHeight="11180" xr2:uid="{122630C5-77A4-D449-8A1A-052F0B5B4F44}"/>
   </bookViews>
   <sheets>
     <sheet name="ERC_SpD_spatial_registration_an" sheetId="1" r:id="rId1"/>
@@ -136,9 +136,6 @@
     <t>Oligo.OPALIN.LAMA2/Oligo.OPALIN.SLC5A11/Oligo.OPALIN.LINC01098/Oligo.CPXM2.KANK4</t>
   </si>
   <si>
-    <t>Annotation</t>
-  </si>
-  <si>
     <t>Vasc</t>
   </si>
   <si>
@@ -157,9 +154,6 @@
     <t>LD</t>
   </si>
   <si>
-    <t>Order</t>
-  </si>
-  <si>
     <t>WMuf</t>
   </si>
   <si>
@@ -194,6 +188,12 @@
   </si>
   <si>
     <t>L3_Inhib</t>
+  </si>
+  <si>
+    <t>anno</t>
+  </si>
+  <si>
+    <t>order</t>
   </si>
 </sst>
 </file>
@@ -1083,13 +1083,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F1" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="G1" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1106,13 +1106,13 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -1129,13 +1129,13 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1152,13 +1152,13 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1175,13 +1175,13 @@
         <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F5">
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1198,13 +1198,13 @@
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6">
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -1221,13 +1221,13 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F7">
         <v>5</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -1244,13 +1244,13 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F8">
         <v>6</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1267,13 +1267,13 @@
         <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F9">
         <v>7</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1290,7 +1290,7 @@
         <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F10">
         <v>8</v>

</xml_diff>